<commit_message>
feat(paie): bulletin de paie PDF par salarié + contre-passation GUIDÉE scellée Evidence — extourne miroir exact (INV-007), re-clôture corrigée -R2 (unicité applicative INV-PAIE), estampille ANNULÉ sur bulletins du run REVERSED, PAYROLL_REVERSAL→journal PAIE, fix withAuth Response.json→NextResponse.json, re-scellement INV-008 (18/18), harnais 38/38 + régressions 37/63/24/28/35/12/22/32 vertes, démo : 2026-07 POSTED · 2026-08 REVERSED · 2026-08-R2 POSTED
</commit_message>
<xml_diff>
--- a/scripts/out_syscohada/balance_ci.xlsx
+++ b/scripts/out_syscohada/balance_ci.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>YAHRIA BUSINESS OS — ÉTATS FINANCIERS SYSCOHADA (SYSTÈME NORMAL)</t>
   </si>
@@ -52,6 +52,24 @@
     <t>Clients</t>
   </si>
   <si>
+    <t>4221</t>
+  </si>
+  <si>
+    <t>Personnel, rémunérations dues</t>
+  </si>
+  <si>
+    <t>4311</t>
+  </si>
+  <si>
+    <t>Sécurité sociale</t>
+  </si>
+  <si>
+    <t>4321</t>
+  </si>
+  <si>
+    <t>État, impôts sur les rémunérations</t>
+  </si>
+  <si>
     <t>4431</t>
   </si>
   <si>
@@ -73,6 +91,12 @@
     <t>Banques (SGCI)</t>
   </si>
   <si>
+    <t>5211</t>
+  </si>
+  <si>
+    <t>Banques</t>
+  </si>
+  <si>
     <t>5212</t>
   </si>
   <si>
@@ -116,6 +140,30 @@
   </si>
   <si>
     <t>Charges de personnel</t>
+  </si>
+  <si>
+    <t>6611</t>
+  </si>
+  <si>
+    <t>Salaires des ouvriers</t>
+  </si>
+  <si>
+    <t>6612</t>
+  </si>
+  <si>
+    <t>Salaires des employés</t>
+  </si>
+  <si>
+    <t>6613</t>
+  </si>
+  <si>
+    <t>Salaires des chefs d’exploitation et de main-d’œuvre</t>
+  </si>
+  <si>
+    <t>6641</t>
+  </si>
+  <si>
+    <t>Cotisations sociales patronales</t>
   </si>
   <si>
     <t>CLASSE 7 — Comptes de produits</t>
@@ -596,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -706,16 +754,16 @@
         <v>4</v>
       </c>
       <c r="D8" s="6">
-        <v>0</v>
+        <v>15025880</v>
       </c>
       <c r="E8" s="6">
-        <v>1155420</v>
+        <v>15025880</v>
       </c>
       <c r="F8" s="6">
         <v>0</v>
       </c>
       <c r="G8" s="6">
-        <v>1155420</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,150 +777,162 @@
         <v>4</v>
       </c>
       <c r="D9" s="6">
-        <v>935100</v>
+        <v>799000</v>
       </c>
       <c r="E9" s="6">
-        <v>0</v>
+        <v>2397000</v>
       </c>
       <c r="F9" s="6">
-        <v>935100</v>
+        <v>0</v>
       </c>
       <c r="G9" s="6">
-        <v>0</v>
+        <v>1598000</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10" s="6">
+        <v>225780</v>
+      </c>
+      <c r="E10" s="6">
+        <v>677340</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>451560</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11" s="6">
-        <v>808300</v>
+        <v>0</v>
       </c>
       <c r="E11" s="6">
-        <v>10380100</v>
+        <v>1155420</v>
       </c>
       <c r="F11" s="6">
         <v>0</v>
       </c>
       <c r="G11" s="6">
-        <v>9571800</v>
+        <v>1155420</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12" s="6">
+        <v>935100</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
+        <v>935100</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14">
         <v>5</v>
       </c>
-      <c r="D12" s="6">
-        <v>545750</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6">
-        <v>545750</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13">
-        <v>5</v>
-      </c>
-      <c r="D13" s="6">
-        <v>1562320</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="6">
-        <v>1562320</v>
-      </c>
-      <c r="G13" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="D14" s="6">
+        <v>808300</v>
+      </c>
+      <c r="E14" s="6">
+        <v>10380100</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>9571800</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15" s="6">
-        <v>620000</v>
+        <v>3756470</v>
       </c>
       <c r="E15" s="6">
-        <v>0</v>
+        <v>11269410</v>
       </c>
       <c r="F15" s="6">
-        <v>620000</v>
+        <v>0</v>
       </c>
       <c r="G15" s="6">
-        <v>0</v>
+        <v>7512940</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16" s="6">
-        <v>1690000</v>
+        <v>545750</v>
       </c>
       <c r="E16" s="6">
         <v>0</v>
       </c>
       <c r="F16" s="6">
-        <v>1690000</v>
+        <v>545750</v>
       </c>
       <c r="G16" s="6">
         <v>0</v>
@@ -880,49 +940,37 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17" s="6">
-        <v>2500000</v>
+        <v>1562320</v>
       </c>
       <c r="E17" s="6">
         <v>0</v>
       </c>
       <c r="F17" s="6">
-        <v>2500000</v>
+        <v>1562320</v>
       </c>
       <c r="G17" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C18">
-        <v>6</v>
-      </c>
-      <c r="D18" s="6">
-        <v>385000</v>
-      </c>
-      <c r="E18" s="6">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6">
-        <v>385000</v>
-      </c>
-      <c r="G18" s="6">
-        <v>0</v>
-      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -935,101 +983,285 @@
         <v>6</v>
       </c>
       <c r="D19" s="6">
-        <v>4250000</v>
+        <v>620000</v>
       </c>
       <c r="E19" s="6">
         <v>0</v>
       </c>
       <c r="F19" s="6">
-        <v>4250000</v>
+        <v>620000</v>
       </c>
       <c r="G19" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20" s="6">
+        <v>1690000</v>
+      </c>
+      <c r="E20" s="6">
+        <v>0</v>
+      </c>
+      <c r="F20" s="6">
+        <v>1690000</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>2500000</v>
       </c>
       <c r="E21" s="6">
-        <v>4414000</v>
+        <v>0</v>
       </c>
       <c r="F21" s="6">
-        <v>0</v>
+        <v>2500000</v>
       </c>
       <c r="G21" s="6">
-        <v>4414000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22" s="6">
+        <v>385000</v>
+      </c>
+      <c r="E22" s="6">
+        <v>0</v>
+      </c>
+      <c r="F22" s="6">
+        <v>385000</v>
+      </c>
+      <c r="G22" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23" s="6">
+        <v>4250000</v>
+      </c>
+      <c r="E23" s="6">
+        <v>0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>4250000</v>
+      </c>
+      <c r="G23" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24">
+        <v>6</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1260000</v>
+      </c>
+      <c r="E24" s="6">
+        <v>420000</v>
+      </c>
+      <c r="F24" s="6">
+        <v>840000</v>
+      </c>
+      <c r="G24" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25">
+        <v>6</v>
+      </c>
+      <c r="D25" s="6">
+        <v>7890000</v>
+      </c>
+      <c r="E25" s="6">
+        <v>2630000</v>
+      </c>
+      <c r="F25" s="6">
+        <v>5260000</v>
+      </c>
+      <c r="G25" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26">
+        <v>6</v>
+      </c>
+      <c r="D26" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="E26" s="6">
+        <v>1200000</v>
+      </c>
+      <c r="F26" s="6">
+        <v>2400000</v>
+      </c>
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27">
+        <v>6</v>
+      </c>
+      <c r="D27" s="6">
+        <v>1593750</v>
+      </c>
+      <c r="E27" s="6">
+        <v>531250</v>
+      </c>
+      <c r="F27" s="6">
+        <v>1062500</v>
+      </c>
+      <c r="G27" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29">
         <v>7</v>
       </c>
-      <c r="D22" s="6">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6">
+      <c r="D29" s="6">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6">
+        <v>4414000</v>
+      </c>
+      <c r="F29" s="6">
+        <v>0</v>
+      </c>
+      <c r="G29" s="6">
+        <v>4414000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30">
+        <v>7</v>
+      </c>
+      <c r="D30" s="6">
+        <v>0</v>
+      </c>
+      <c r="E30" s="6">
         <v>2005000</v>
       </c>
-      <c r="F22" s="6">
-        <v>0</v>
-      </c>
-      <c r="G22" s="6">
+      <c r="F30" s="6">
+        <v>0</v>
+      </c>
+      <c r="G30" s="6">
         <v>2005000</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="9">
-        <v>20870890</v>
-      </c>
-      <c r="E23" s="9">
-        <v>20870890</v>
-      </c>
-      <c r="F23" s="9">
-        <v>17146220</v>
-      </c>
-      <c r="G23" s="9">
-        <v>17146220</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>42</v>
+    <row r="31" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="9">
+        <v>55021770</v>
+      </c>
+      <c r="E31" s="9">
+        <v>55021770</v>
+      </c>
+      <c r="F31" s="9">
+        <v>26708720</v>
+      </c>
+      <c r="G31" s="9">
+        <v>26708720</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1038,9 +1270,9 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>